<commit_message>
chore(seed): adiciona relatórios de seed e planilha de mapeamento atualizada
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/normalizacao_dados/CATEGORIA NOVA X CATEGORIA ANTIGA.xlsx
+++ b/normalizacao_dados/CATEGORIA NOVA X CATEGORIA ANTIGA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guilherme.frade\Desktop\Backup Guilherme\BACKUP - Guilherme\BACKUP - Guilherme\Automacao_python\sistema_de_ouvidoria\normalizacao_dados\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos\sistema_de_ouvidoria\normalizacao_dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{892087E7-0B1B-4220-84D6-E1A600C8AB2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1E619C7-DDEA-40DA-82C4-DAF40FB889D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{E44C7F00-188F-48A6-B078-824DDA47D2D2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{E44C7F00-188F-48A6-B078-824DDA47D2D2}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="60">
   <si>
     <t>ACESSIBILIDADE</t>
   </si>
@@ -204,6 +204,18 @@
   </si>
   <si>
     <t>ANTIGAS SUBCATEGORIAS (ASSUNTO)</t>
+  </si>
+  <si>
+    <t>SUPRESSÃO DE HORÁRIO</t>
+  </si>
+  <si>
+    <t>VALOR DA PASSAGEM</t>
+  </si>
+  <si>
+    <t>CRÍTICA À REGULAMENTAÇÃO</t>
+  </si>
+  <si>
+    <t>AUMENTO DE FROTA</t>
   </si>
 </sst>
 </file>
@@ -294,7 +306,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -319,6 +331,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -654,7 +669,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48F34548-9684-42F9-81BF-B15EF804A057}">
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="52.140625" customWidth="1"/>
@@ -932,6 +947,30 @@
         <v>53</v>
       </c>
     </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36" s="9" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B37" s="9" t="s">
+        <v>38</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>